<commit_message>
Se incorpora una ventana final de resumen en la carga masiva
</commit_message>
<xml_diff>
--- a/alumnos_ejemplo.xlsx
+++ b/alumnos_ejemplo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,6 +715,41 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>alumno.error1@usch.cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>alumno.error2@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>alumno.error3@usach.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>alumno.error4@usach.cl.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>alumno.error5@usach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>